<commit_message>
Master TP Done tinggal Formatif nya belum
</commit_message>
<xml_diff>
--- a/public/down/Template_InputSiswa.xlsx
+++ b/public/down/Template_InputSiswa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Indraa\Documents\codingan\SiNilai\public\down\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78AB8BD4-2E29-4E12-8D98-A28D848F8434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EB5C250-37A3-49DB-B720-44E03303745D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5615BEBA-C1D9-49E6-A268-EEAE007A5A71}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{5615BEBA-C1D9-49E6-A268-EEAE007A5A71}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>NIS</t>
   </si>
@@ -79,6 +79,15 @@
   </si>
   <si>
     <t>ALAMAT ORANG TUA</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>A</t>
   </si>
 </sst>
 </file>
@@ -102,7 +111,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -125,6 +134,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -132,7 +152,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -447,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53E4A36D-B9DF-4BD9-93A3-F11422EF4DBE}">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -459,9 +479,12 @@
     <col min="13" max="13" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="1.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="2.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -471,7 +494,7 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -507,7 +530,15 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1"/>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixing new Schema And Newer FIx Core nya belum beres
</commit_message>
<xml_diff>
--- a/public/down/Template_InputSiswa.xlsx
+++ b/public/down/Template_InputSiswa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25330"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Indraa\Documents\codingan\SiNilai\public\down\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Indraaaa\Documents\codingan\app-nilai\public\down\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EB5C250-37A3-49DB-B720-44E03303745D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2E34BE5-2E00-4DB9-A712-1C36F9DE55F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{5615BEBA-C1D9-49E6-A268-EEAE007A5A71}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{5615BEBA-C1D9-49E6-A268-EEAE007A5A71}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>